<commit_message>
Listing errors in Study 2 Video 4
</commit_message>
<xml_diff>
--- a/reference_keys/KEY_Video_4.xlsx
+++ b/reference_keys/KEY_Video_4.xlsx
@@ -3978,7 +3978,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Listing is present: 3+ symbols of same part of speech</t>
+          <t>Listing is Not Present</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4223,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Listing is present: 3+ symbols of same part of speech</t>
+          <t>Listing is Not Present</t>
         </is>
       </c>
     </row>

</xml_diff>